<commit_message>
Added Bulk Upload logic for Product Lines
</commit_message>
<xml_diff>
--- a/CPQ Hierarchy/Master Data.xlsx
+++ b/CPQ Hierarchy/Master Data.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ddg15\Documents\UiPath\CPQ Automation\CPQ Hierarchy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32864A26-D2FB-4983-9D13-E2B72DE30052}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1876737C-4F7B-4DD9-BB2D-CC45DB749AE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{46C2E97C-D120-49E3-B927-F7CE7436F631}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{46C2E97C-D120-49E3-B927-F7CE7436F631}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="37">
   <si>
     <t>Prod Family</t>
   </si>
@@ -100,6 +101,51 @@
   </si>
   <si>
     <t>Domestic~International</t>
+  </si>
+  <si>
+    <t>Product Lines</t>
+  </si>
+  <si>
+    <t>Hatchbacks</t>
+  </si>
+  <si>
+    <t>Sedans</t>
+  </si>
+  <si>
+    <t>Jets</t>
+  </si>
+  <si>
+    <t>Product Line Attributes</t>
+  </si>
+  <si>
+    <t>PL Attribute Type</t>
+  </si>
+  <si>
+    <t>PL Attribute Data Type</t>
+  </si>
+  <si>
+    <t>PL Attribute Values</t>
+  </si>
+  <si>
+    <t>Radio</t>
+  </si>
+  <si>
+    <t>Tyre Size</t>
+  </si>
+  <si>
+    <t>ADAS Features</t>
+  </si>
+  <si>
+    <t>13~14~15</t>
+  </si>
+  <si>
+    <t>ABS~EBD~Collission Warning~Cruise Control</t>
+  </si>
+  <si>
+    <t>Multi Select Menu</t>
+  </si>
+  <si>
+    <t>Seating Capacity</t>
   </si>
 </sst>
 </file>
@@ -202,7 +248,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -220,6 +266,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -660,4 +718,116 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6BDED2D-06AB-4909-B7B9-0CD32AFA755E}">
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.85546875" customWidth="1"/>
+    <col min="5" max="5" width="37.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="40.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" s="8"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="7"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="7"/>
+      <c r="B4" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" s="8"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="A2:A4"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Added Bulk Upload logic for Attributes
</commit_message>
<xml_diff>
--- a/CPQ Hierarchy/Master Data.xlsx
+++ b/CPQ Hierarchy/Master Data.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ddg15\Documents\UiPath\CPQ Automation\CPQ Hierarchy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1876737C-4F7B-4DD9-BB2D-CC45DB749AE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D505738D-CE98-41C6-B89F-691EA02524CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{46C2E97C-D120-49E3-B927-F7CE7436F631}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{46C2E97C-D120-49E3-B927-F7CE7436F631}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Product Family" sheetId="1" r:id="rId1"/>
+    <sheet name="Product Line" sheetId="2" r:id="rId2"/>
+    <sheet name="Model" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="64">
   <si>
     <t>Prod Family</t>
   </si>
@@ -146,13 +147,94 @@
   </si>
   <si>
     <t>Seating Capacity</t>
+  </si>
+  <si>
+    <t>Models</t>
+  </si>
+  <si>
+    <t>Alto</t>
+  </si>
+  <si>
+    <t>Altroz</t>
+  </si>
+  <si>
+    <t>Model Attributes</t>
+  </si>
+  <si>
+    <t>Model Attribute Data Type</t>
+  </si>
+  <si>
+    <t>Model Attribute Type</t>
+  </si>
+  <si>
+    <t>Model Attribute Values</t>
+  </si>
+  <si>
+    <t>Car Model</t>
+  </si>
+  <si>
+    <t>Air Conditioning</t>
+  </si>
+  <si>
+    <t>Infotainment</t>
+  </si>
+  <si>
+    <t>Airbus</t>
+  </si>
+  <si>
+    <t>Boeing</t>
+  </si>
+  <si>
+    <t>Design</t>
+  </si>
+  <si>
+    <t>Controls</t>
+  </si>
+  <si>
+    <t>Comfort Class</t>
+  </si>
+  <si>
+    <t>Virtus</t>
+  </si>
+  <si>
+    <t>Wheel Design</t>
+  </si>
+  <si>
+    <t>Private Bus</t>
+  </si>
+  <si>
+    <t>Public Bus</t>
+  </si>
+  <si>
+    <t>Distance</t>
+  </si>
+  <si>
+    <t>Number of Trips</t>
+  </si>
+  <si>
+    <t>LXI~VXI</t>
+  </si>
+  <si>
+    <t>Steel~Alloy Wheels</t>
+  </si>
+  <si>
+    <t>Business~Semi-Business</t>
+  </si>
+  <si>
+    <t>Volvo</t>
+  </si>
+  <si>
+    <t>State Transport</t>
+  </si>
+  <si>
+    <t>2~3~4</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -171,6 +253,14 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -248,7 +338,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -259,6 +349,33 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -268,16 +385,16 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -621,7 +738,7 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="13" t="s">
         <v>5</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -636,7 +753,7 @@
       <c r="E2" s="2"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="5"/>
+      <c r="A3" s="14"/>
       <c r="B3" s="2" t="s">
         <v>12</v>
       </c>
@@ -651,7 +768,7 @@
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="13" t="s">
         <v>6</v>
       </c>
       <c r="B4" s="2" t="s">
@@ -668,7 +785,7 @@
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="6"/>
+      <c r="A5" s="15"/>
       <c r="B5" s="2" t="s">
         <v>16</v>
       </c>
@@ -683,7 +800,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="5"/>
+      <c r="A6" s="14"/>
       <c r="B6" s="2" t="s">
         <v>17</v>
       </c>
@@ -702,10 +819,10 @@
       <c r="B7" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="12" t="s">
         <v>10</v>
       </c>
       <c r="E7" s="2"/>
@@ -722,7 +839,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6BDED2D-06AB-4909-B7B9-0CD32AFA755E}">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.42578125" bestFit="1" customWidth="1"/>
@@ -754,13 +871,13 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="5" t="s">
         <v>30</v>
       </c>
       <c r="D2" s="2" t="s">
@@ -769,12 +886,12 @@
       <c r="E2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="8"/>
+      <c r="F2" s="5"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="7"/>
-      <c r="B3" s="9"/>
-      <c r="C3" s="8" t="s">
+      <c r="A3" s="17"/>
+      <c r="B3" s="16"/>
+      <c r="C3" s="5" t="s">
         <v>31</v>
       </c>
       <c r="D3" s="2" t="s">
@@ -788,11 +905,11 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="7"/>
-      <c r="B4" s="8" t="s">
+      <c r="A4" s="17"/>
+      <c r="B4" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="5" t="s">
         <v>32</v>
       </c>
       <c r="D4" s="2" t="s">
@@ -806,13 +923,13 @@
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="7" t="s">
         <v>36</v>
       </c>
       <c r="D5" s="2" t="s">
@@ -821,13 +938,261 @@
       <c r="E5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="F5" s="8"/>
+      <c r="F5" s="5"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="C6" s="6"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
+      <c r="F6" s="6"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="19"/>
+      <c r="B7" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="A2:A4"/>
+    <mergeCell ref="A6:A7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{002AB8A0-9CDC-4CC0-8DFC-F2BA8853CB21}">
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="25" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="F1" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="16" t="s">
+        <v>38</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="E2" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="15"/>
+      <c r="B3" s="16"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G3" s="4"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="15"/>
+      <c r="B4" s="16"/>
+      <c r="C4" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4" s="4"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="14"/>
+      <c r="B5" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="E5" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="G5" s="11" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>47</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="G6" s="6"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="16"/>
+      <c r="B7" s="16"/>
+      <c r="C7" s="16"/>
+      <c r="D7" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="G7" s="6"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="16"/>
+      <c r="B8" s="16"/>
+      <c r="C8" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="G8" s="11" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="G9" s="6"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="19"/>
+      <c r="B10" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="D10" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F10" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>63</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A6:A8"/>
+    <mergeCell ref="B6:B8"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="B2:B4"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>